<commit_message>
Update reproducibility repository package
</commit_message>
<xml_diff>
--- a/tables/S2_Table_cancer_normal_evidence_table.xlsx
+++ b/tables/S2_Table_cancer_normal_evidence_table.xlsx
@@ -1179,21 +1179,17 @@
           <t>6</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0.486</t>
-        </is>
+      <c r="L2" t="n">
+        <v>0.424</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>lower PRISM cancer-preservation risk</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>PRISM PC penalty=0.486; lower PRISM cancer-preservation risk</t>
+          <t>PRISM P_C descriptor=0.424; lower PRISM cancer-preservation risk</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -1248,7 +1244,6 @@
           <t>strong cytoprotection can imply high cancer-preservation penalty in stressed cancer cells</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -1264,21 +1259,17 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0.962</t>
-        </is>
+      <c r="L3" t="n">
+        <v>0.997</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>high PRISM cancer-preservation risk</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>PRISM PC penalty=0.962; high PRISM cancer-preservation risk</t>
+          <t>PRISM P_C descriptor=0.997; high PRISM cancer-preservation risk</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -1333,7 +1324,6 @@
           <t>clinical evidence mixed; mechanism is metabolic/AGE/NF-κB, not simple antioxidant</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -1349,21 +1339,17 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>0.463</t>
-        </is>
+      <c r="L4" t="n">
+        <v>0.527</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
           <t>lower PRISM cancer-preservation risk</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>PRISM PC penalty=0.463; lower PRISM cancer-preservation risk</t>
+          <t>PRISM P_C descriptor=0.527; lower PRISM cancer-preservation risk</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1418,7 +1404,6 @@
           <t>less direct human normal-cell evidence than Trolox/EGT</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -1434,21 +1419,17 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>0.783</t>
-        </is>
+      <c r="L5" t="n">
+        <v>0.894</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
           <t>high PRISM cancer-preservation risk</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>PRISM PC penalty=0.783; high PRISM cancer-preservation risk</t>
+          <t>PRISM P_C descriptor=0.894; high PRISM cancer-preservation risk</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1483,10 +1464,6 @@
           <t>glucocorticoid representative</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>1.0</t>
@@ -1507,14 +1484,11 @@
           <t>17</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -1552,11 +1526,6 @@
           <t>glucocorticoid representative</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -1572,14 +1541,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -1617,10 +1583,6 @@
           <t>glucocorticoid representative</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>1.0</t>
@@ -1641,14 +1603,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -1686,11 +1645,6 @@
           <t>CHK / DDR checkpoint</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -1706,7 +1660,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -1759,11 +1712,6 @@
           <t>CHK / DDR checkpoint</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -1779,7 +1727,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -1832,10 +1779,6 @@
           <t>CHK / DDR checkpoint</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>1.0</t>
@@ -1856,7 +1799,6 @@
           <t>9</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -1909,11 +1851,6 @@
           <t>CHK / DDR checkpoint</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -1929,7 +1866,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -1982,11 +1918,6 @@
           <t>HSP / proteostasis</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -2002,7 +1933,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2055,10 +1985,6 @@
           <t>HSP / proteostasis</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>1.0</t>
@@ -2079,7 +2005,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2132,11 +2057,6 @@
           <t>HSP / proteostasis</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -2152,7 +2072,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2205,11 +2124,6 @@
           <t>KIF11 / kinesin / spindle</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -2225,7 +2139,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2278,11 +2191,6 @@
           <t>KIF11 / kinesin / spindle</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -2298,7 +2206,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2351,11 +2258,6 @@
           <t>KIF11 / kinesin / spindle</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -2371,7 +2273,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2424,11 +2325,6 @@
           <t>KIF11 / kinesin / spindle</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -2444,7 +2340,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2497,10 +2392,6 @@
           <t>PLK / Aurora / mitotic checkpoint</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>1.0</t>
@@ -2521,7 +2412,6 @@
           <t>24</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2574,10 +2464,6 @@
           <t>PLK / Aurora / mitotic checkpoint</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>1.0</t>
@@ -2598,7 +2484,6 @@
           <t>14</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2651,11 +2536,6 @@
           <t>PLK / Aurora / mitotic checkpoint</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -2671,7 +2551,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2724,11 +2603,6 @@
           <t>PLK / Aurora / mitotic checkpoint</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>TN missing / insufficient curated ChEMBL normal-like data</t>
@@ -2744,7 +2618,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>not assessed as repair-preservation candidate</t>
@@ -2918,12 +2791,9 @@
           <t>0.688</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.783</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>0.894</v>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>0.56</t>
@@ -2939,10 +2809,8 @@
           <t>0.36</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>-0.335</t>
-        </is>
+      <c r="N2" t="n">
+        <v>-0.446</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -2996,12 +2864,9 @@
           <t>0.688</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.486</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>0.424</v>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>0.56</t>
@@ -3017,10 +2882,8 @@
           <t>0.36</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0.082</t>
-        </is>
+      <c r="N3" t="n">
+        <v>0.144</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -3074,12 +2937,9 @@
           <t>0.688</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.463</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>0.527</v>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>0.56</t>
@@ -3095,10 +2955,8 @@
           <t>0.36</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>-0.075</t>
-        </is>
+      <c r="N4" t="n">
+        <v>-0.139</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -3152,12 +3010,9 @@
           <t>0.688</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>0.962</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>0.997</v>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>0.56</t>
@@ -3173,10 +3028,8 @@
           <t>0.36</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>-0.334</t>
-        </is>
+      <c r="N5" t="n">
+        <v>-0.369</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -3230,10 +3083,8 @@
           <t>0.76</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0.783</t>
-        </is>
+      <c r="I6" t="n">
+        <v>0.894</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -3255,10 +3106,8 @@
           <t>0.36</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>-0.703</t>
-        </is>
+      <c r="N6" t="n">
+        <v>-0.8139999999999999</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>

</xml_diff>